<commit_message>
Refactor verdict classification: merge 'MISLEADING' into 'PARTIALLY TRUE'
- Updated model to remove 'MISLEADING' verdict, folding it into 'PARTIALLY TRUE' for backward compatibility.
- Adjusted metrics and evaluation files to reflect the new verdict structure.
- Modified confusion matrices, metrics calculations, and predictions to accommodate the change.
- Updated tests to ensure correct handling of the new verdict classification.
- Revised documentation and comments to clarify the new verdict definitions and implications.
</commit_message>
<xml_diff>
--- a/fact_checker_evaluation_dataset.xlsx
+++ b/fact_checker_evaluation_dataset.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evaluation Dataset" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verdict Definitions" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Evaluation Dataset'!$A$1:$G$101</definedName>
@@ -492,10 +493,6 @@
           <t>TRUE</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -511,10 +508,6 @@
           <t>TRUE</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -530,10 +523,6 @@
           <t>TRUE</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -549,10 +538,6 @@
           <t>TRUE</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -568,10 +553,6 @@
           <t>TRUE</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -587,10 +568,6 @@
           <t>TRUE</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -606,10 +583,6 @@
           <t>TRUE</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -625,10 +598,6 @@
           <t>TRUE</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -644,10 +613,6 @@
           <t>TRUE</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -663,10 +628,6 @@
           <t>TRUE</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -682,10 +643,6 @@
           <t>TRUE</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -701,10 +658,6 @@
           <t>TRUE</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -720,10 +673,6 @@
           <t>TRUE</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -739,10 +688,6 @@
           <t>TRUE</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -758,10 +703,6 @@
           <t>TRUE</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -777,10 +718,6 @@
           <t>TRUE</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -796,10 +733,6 @@
           <t>TRUE</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -815,10 +748,6 @@
           <t>TRUE</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -834,10 +763,6 @@
           <t>TRUE</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -853,10 +778,6 @@
           <t>TRUE</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -872,10 +793,6 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -891,10 +808,6 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -910,10 +823,6 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -929,10 +838,6 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -948,10 +853,6 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -967,10 +868,6 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -986,10 +883,6 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1005,10 +898,6 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1024,10 +913,6 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1043,10 +928,6 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1062,10 +943,6 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1081,10 +958,6 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1100,10 +973,6 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr"/>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1119,10 +988,6 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1138,10 +1003,6 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1157,10 +1018,6 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr"/>
-      <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1176,10 +1033,6 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr"/>
-      <c r="E38" t="inlineStr"/>
-      <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1195,10 +1048,6 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr"/>
-      <c r="E39" t="inlineStr"/>
-      <c r="F39" t="inlineStr"/>
-      <c r="G39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -1214,10 +1063,6 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr"/>
-      <c r="E40" t="inlineStr"/>
-      <c r="F40" t="inlineStr"/>
-      <c r="G40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -1233,10 +1078,6 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr"/>
-      <c r="E41" t="inlineStr"/>
-      <c r="F41" t="inlineStr"/>
-      <c r="G41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -1252,10 +1093,6 @@
           <t>PARTIALLY TRUE</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr"/>
-      <c r="E42" t="inlineStr"/>
-      <c r="F42" t="inlineStr"/>
-      <c r="G42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -1271,10 +1108,6 @@
           <t>PARTIALLY TRUE</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr"/>
-      <c r="E43" t="inlineStr"/>
-      <c r="F43" t="inlineStr"/>
-      <c r="G43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -1290,10 +1123,6 @@
           <t>PARTIALLY TRUE</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr"/>
-      <c r="E44" t="inlineStr"/>
-      <c r="F44" t="inlineStr"/>
-      <c r="G44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -1309,10 +1138,6 @@
           <t>PARTIALLY TRUE</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr"/>
-      <c r="E45" t="inlineStr"/>
-      <c r="F45" t="inlineStr"/>
-      <c r="G45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -1328,10 +1153,6 @@
           <t>PARTIALLY TRUE</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr"/>
-      <c r="E46" t="inlineStr"/>
-      <c r="F46" t="inlineStr"/>
-      <c r="G46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -1347,10 +1168,6 @@
           <t>PARTIALLY TRUE</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr"/>
-      <c r="E47" t="inlineStr"/>
-      <c r="F47" t="inlineStr"/>
-      <c r="G47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -1366,10 +1183,6 @@
           <t>PARTIALLY TRUE</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr"/>
-      <c r="E48" t="inlineStr"/>
-      <c r="F48" t="inlineStr"/>
-      <c r="G48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -1385,10 +1198,6 @@
           <t>PARTIALLY TRUE</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr"/>
-      <c r="E49" t="inlineStr"/>
-      <c r="F49" t="inlineStr"/>
-      <c r="G49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -1404,10 +1213,6 @@
           <t>PARTIALLY TRUE</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr"/>
-      <c r="E50" t="inlineStr"/>
-      <c r="F50" t="inlineStr"/>
-      <c r="G50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -1423,10 +1228,6 @@
           <t>PARTIALLY TRUE</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr"/>
-      <c r="E51" t="inlineStr"/>
-      <c r="F51" t="inlineStr"/>
-      <c r="G51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -1442,10 +1243,6 @@
           <t>PARTIALLY TRUE</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr"/>
-      <c r="E52" t="inlineStr"/>
-      <c r="F52" t="inlineStr"/>
-      <c r="G52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -1461,10 +1258,6 @@
           <t>PARTIALLY TRUE</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr"/>
-      <c r="E53" t="inlineStr"/>
-      <c r="F53" t="inlineStr"/>
-      <c r="G53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -1480,10 +1273,6 @@
           <t>PARTIALLY TRUE</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr"/>
-      <c r="E54" t="inlineStr"/>
-      <c r="F54" t="inlineStr"/>
-      <c r="G54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -1499,10 +1288,6 @@
           <t>PARTIALLY TRUE</t>
         </is>
       </c>
-      <c r="D55" t="inlineStr"/>
-      <c r="E55" t="inlineStr"/>
-      <c r="F55" t="inlineStr"/>
-      <c r="G55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -1518,10 +1303,6 @@
           <t>PARTIALLY TRUE</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr"/>
-      <c r="E56" t="inlineStr"/>
-      <c r="F56" t="inlineStr"/>
-      <c r="G56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -1537,10 +1318,6 @@
           <t>PARTIALLY TRUE</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr"/>
-      <c r="E57" t="inlineStr"/>
-      <c r="F57" t="inlineStr"/>
-      <c r="G57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -1556,10 +1333,6 @@
           <t>PARTIALLY TRUE</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr"/>
-      <c r="E58" t="inlineStr"/>
-      <c r="F58" t="inlineStr"/>
-      <c r="G58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -1575,10 +1348,6 @@
           <t>PARTIALLY TRUE</t>
         </is>
       </c>
-      <c r="D59" t="inlineStr"/>
-      <c r="E59" t="inlineStr"/>
-      <c r="F59" t="inlineStr"/>
-      <c r="G59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -1594,10 +1363,6 @@
           <t>PARTIALLY TRUE</t>
         </is>
       </c>
-      <c r="D60" t="inlineStr"/>
-      <c r="E60" t="inlineStr"/>
-      <c r="F60" t="inlineStr"/>
-      <c r="G60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -1613,10 +1378,6 @@
           <t>PARTIALLY TRUE</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr"/>
-      <c r="E61" t="inlineStr"/>
-      <c r="F61" t="inlineStr"/>
-      <c r="G61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -1629,13 +1390,9 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>MISLEADING</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr"/>
-      <c r="E62" t="inlineStr"/>
-      <c r="F62" t="inlineStr"/>
-      <c r="G62" t="inlineStr"/>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -1648,13 +1405,9 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>MISLEADING</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr"/>
-      <c r="E63" t="inlineStr"/>
-      <c r="F63" t="inlineStr"/>
-      <c r="G63" t="inlineStr"/>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -1667,13 +1420,9 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>MISLEADING</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr"/>
-      <c r="E64" t="inlineStr"/>
-      <c r="F64" t="inlineStr"/>
-      <c r="G64" t="inlineStr"/>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -1686,13 +1435,9 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>MISLEADING</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr"/>
-      <c r="E65" t="inlineStr"/>
-      <c r="F65" t="inlineStr"/>
-      <c r="G65" t="inlineStr"/>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -1705,13 +1450,9 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>MISLEADING</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr"/>
-      <c r="E66" t="inlineStr"/>
-      <c r="F66" t="inlineStr"/>
-      <c r="G66" t="inlineStr"/>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -1724,13 +1465,9 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>MISLEADING</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr"/>
-      <c r="E67" t="inlineStr"/>
-      <c r="F67" t="inlineStr"/>
-      <c r="G67" t="inlineStr"/>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -1743,13 +1480,9 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>MISLEADING</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr"/>
-      <c r="E68" t="inlineStr"/>
-      <c r="F68" t="inlineStr"/>
-      <c r="G68" t="inlineStr"/>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -1762,13 +1495,9 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>MISLEADING</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr"/>
-      <c r="E69" t="inlineStr"/>
-      <c r="F69" t="inlineStr"/>
-      <c r="G69" t="inlineStr"/>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -1781,13 +1510,9 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>MISLEADING</t>
-        </is>
-      </c>
-      <c r="D70" t="inlineStr"/>
-      <c r="E70" t="inlineStr"/>
-      <c r="F70" t="inlineStr"/>
-      <c r="G70" t="inlineStr"/>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -1800,13 +1525,9 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>MISLEADING</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr"/>
-      <c r="E71" t="inlineStr"/>
-      <c r="F71" t="inlineStr"/>
-      <c r="G71" t="inlineStr"/>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -1819,13 +1540,9 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>MISLEADING</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr"/>
-      <c r="E72" t="inlineStr"/>
-      <c r="F72" t="inlineStr"/>
-      <c r="G72" t="inlineStr"/>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -1838,13 +1555,9 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>MISLEADING</t>
-        </is>
-      </c>
-      <c r="D73" t="inlineStr"/>
-      <c r="E73" t="inlineStr"/>
-      <c r="F73" t="inlineStr"/>
-      <c r="G73" t="inlineStr"/>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -1857,13 +1570,9 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>MISLEADING</t>
-        </is>
-      </c>
-      <c r="D74" t="inlineStr"/>
-      <c r="E74" t="inlineStr"/>
-      <c r="F74" t="inlineStr"/>
-      <c r="G74" t="inlineStr"/>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -1876,13 +1585,9 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>MISLEADING</t>
-        </is>
-      </c>
-      <c r="D75" t="inlineStr"/>
-      <c r="E75" t="inlineStr"/>
-      <c r="F75" t="inlineStr"/>
-      <c r="G75" t="inlineStr"/>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -1895,13 +1600,9 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>MISLEADING</t>
-        </is>
-      </c>
-      <c r="D76" t="inlineStr"/>
-      <c r="E76" t="inlineStr"/>
-      <c r="F76" t="inlineStr"/>
-      <c r="G76" t="inlineStr"/>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -1914,13 +1615,9 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>MISLEADING</t>
-        </is>
-      </c>
-      <c r="D77" t="inlineStr"/>
-      <c r="E77" t="inlineStr"/>
-      <c r="F77" t="inlineStr"/>
-      <c r="G77" t="inlineStr"/>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -1933,13 +1630,9 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>MISLEADING</t>
-        </is>
-      </c>
-      <c r="D78" t="inlineStr"/>
-      <c r="E78" t="inlineStr"/>
-      <c r="F78" t="inlineStr"/>
-      <c r="G78" t="inlineStr"/>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -1952,13 +1645,9 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>MISLEADING</t>
-        </is>
-      </c>
-      <c r="D79" t="inlineStr"/>
-      <c r="E79" t="inlineStr"/>
-      <c r="F79" t="inlineStr"/>
-      <c r="G79" t="inlineStr"/>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -1971,13 +1660,9 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>MISLEADING</t>
-        </is>
-      </c>
-      <c r="D80" t="inlineStr"/>
-      <c r="E80" t="inlineStr"/>
-      <c r="F80" t="inlineStr"/>
-      <c r="G80" t="inlineStr"/>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -1990,13 +1675,9 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>MISLEADING</t>
-        </is>
-      </c>
-      <c r="D81" t="inlineStr"/>
-      <c r="E81" t="inlineStr"/>
-      <c r="F81" t="inlineStr"/>
-      <c r="G81" t="inlineStr"/>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -2012,10 +1693,6 @@
           <t>UNVERIFIABLE</t>
         </is>
       </c>
-      <c r="D82" t="inlineStr"/>
-      <c r="E82" t="inlineStr"/>
-      <c r="F82" t="inlineStr"/>
-      <c r="G82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -2031,10 +1708,6 @@
           <t>UNVERIFIABLE</t>
         </is>
       </c>
-      <c r="D83" t="inlineStr"/>
-      <c r="E83" t="inlineStr"/>
-      <c r="F83" t="inlineStr"/>
-      <c r="G83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -2050,10 +1723,6 @@
           <t>UNVERIFIABLE</t>
         </is>
       </c>
-      <c r="D84" t="inlineStr"/>
-      <c r="E84" t="inlineStr"/>
-      <c r="F84" t="inlineStr"/>
-      <c r="G84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -2069,10 +1738,6 @@
           <t>UNVERIFIABLE</t>
         </is>
       </c>
-      <c r="D85" t="inlineStr"/>
-      <c r="E85" t="inlineStr"/>
-      <c r="F85" t="inlineStr"/>
-      <c r="G85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -2088,10 +1753,6 @@
           <t>UNVERIFIABLE</t>
         </is>
       </c>
-      <c r="D86" t="inlineStr"/>
-      <c r="E86" t="inlineStr"/>
-      <c r="F86" t="inlineStr"/>
-      <c r="G86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -2107,10 +1768,6 @@
           <t>UNVERIFIABLE</t>
         </is>
       </c>
-      <c r="D87" t="inlineStr"/>
-      <c r="E87" t="inlineStr"/>
-      <c r="F87" t="inlineStr"/>
-      <c r="G87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -2126,10 +1783,6 @@
           <t>UNVERIFIABLE</t>
         </is>
       </c>
-      <c r="D88" t="inlineStr"/>
-      <c r="E88" t="inlineStr"/>
-      <c r="F88" t="inlineStr"/>
-      <c r="G88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -2145,10 +1798,6 @@
           <t>UNVERIFIABLE</t>
         </is>
       </c>
-      <c r="D89" t="inlineStr"/>
-      <c r="E89" t="inlineStr"/>
-      <c r="F89" t="inlineStr"/>
-      <c r="G89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -2164,10 +1813,6 @@
           <t>UNVERIFIABLE</t>
         </is>
       </c>
-      <c r="D90" t="inlineStr"/>
-      <c r="E90" t="inlineStr"/>
-      <c r="F90" t="inlineStr"/>
-      <c r="G90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -2183,10 +1828,6 @@
           <t>UNVERIFIABLE</t>
         </is>
       </c>
-      <c r="D91" t="inlineStr"/>
-      <c r="E91" t="inlineStr"/>
-      <c r="F91" t="inlineStr"/>
-      <c r="G91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -2202,10 +1843,6 @@
           <t>UNVERIFIABLE</t>
         </is>
       </c>
-      <c r="D92" t="inlineStr"/>
-      <c r="E92" t="inlineStr"/>
-      <c r="F92" t="inlineStr"/>
-      <c r="G92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -2221,10 +1858,6 @@
           <t>UNVERIFIABLE</t>
         </is>
       </c>
-      <c r="D93" t="inlineStr"/>
-      <c r="E93" t="inlineStr"/>
-      <c r="F93" t="inlineStr"/>
-      <c r="G93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -2240,10 +1873,6 @@
           <t>UNVERIFIABLE</t>
         </is>
       </c>
-      <c r="D94" t="inlineStr"/>
-      <c r="E94" t="inlineStr"/>
-      <c r="F94" t="inlineStr"/>
-      <c r="G94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -2259,10 +1888,6 @@
           <t>UNVERIFIABLE</t>
         </is>
       </c>
-      <c r="D95" t="inlineStr"/>
-      <c r="E95" t="inlineStr"/>
-      <c r="F95" t="inlineStr"/>
-      <c r="G95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -2278,10 +1903,6 @@
           <t>UNVERIFIABLE</t>
         </is>
       </c>
-      <c r="D96" t="inlineStr"/>
-      <c r="E96" t="inlineStr"/>
-      <c r="F96" t="inlineStr"/>
-      <c r="G96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -2297,10 +1918,6 @@
           <t>UNVERIFIABLE</t>
         </is>
       </c>
-      <c r="D97" t="inlineStr"/>
-      <c r="E97" t="inlineStr"/>
-      <c r="F97" t="inlineStr"/>
-      <c r="G97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -2316,10 +1933,6 @@
           <t>UNVERIFIABLE</t>
         </is>
       </c>
-      <c r="D98" t="inlineStr"/>
-      <c r="E98" t="inlineStr"/>
-      <c r="F98" t="inlineStr"/>
-      <c r="G98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -2335,10 +1948,6 @@
           <t>UNVERIFIABLE</t>
         </is>
       </c>
-      <c r="D99" t="inlineStr"/>
-      <c r="E99" t="inlineStr"/>
-      <c r="F99" t="inlineStr"/>
-      <c r="G99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -2354,10 +1963,6 @@
           <t>UNVERIFIABLE</t>
         </is>
       </c>
-      <c r="D100" t="inlineStr"/>
-      <c r="E100" t="inlineStr"/>
-      <c r="F100" t="inlineStr"/>
-      <c r="G100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -2373,10 +1978,6 @@
           <t>UNVERIFIABLE</t>
         </is>
       </c>
-      <c r="D101" t="inlineStr"/>
-      <c r="E101" t="inlineStr"/>
-      <c r="F101" t="inlineStr"/>
-      <c r="G101" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:G101"/>
@@ -2497,4 +2098,82 @@
   <autoFilter ref="A1:B8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="110" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Verdict</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Definition</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Relevant evidence clearly confirms the claim as stated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Relevant evidence clearly contradicts the claim.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Mixed evidence: some elements are accurate, but the claim overstates, omits key context, holds only under specific conditions, or creates a false impression (includes former MISLEADING).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>UNVERIFIABLE</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>No relevant sources, or insufficient information to judge.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Refactor verdict system to remove 'PARTIALLY TRUE' and transition to a 3-class model
- Introduced a new predictions dataset for evaluation with updated claims and predictions.
- Updated confusion matrix to reflect the removal of 'PARTIALLY TRUE' verdict.
- Adjusted metrics calculations and JSON output to align with the new 3-class verdict system.
- Modified prediction results to remove 'PARTIALLY TRUE' and ensure consistency across evaluation files.
- Refactored evaluation scripts to eliminate legacy verdict aliases and streamline verdict processing.
- Updated tests to validate the new 3-class system and ensure proper handling of verdicts.
- Removed references to 'PARTIALLY TRUE' from scoring and UI components.
</commit_message>
<xml_diff>
--- a/fact_checker_evaluation_dataset.xlsx
+++ b/fact_checker_evaluation_dataset.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evaluation Dataset" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verdict Definitions" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relabel Log" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Evaluation Dataset'!$A$1:$G$101</definedName>
@@ -1090,7 +1091,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>PARTIALLY TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -1105,7 +1106,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>PARTIALLY TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -1120,7 +1121,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>PARTIALLY TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -1135,7 +1136,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>PARTIALLY TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -1150,7 +1151,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>PARTIALLY TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -1165,7 +1166,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>PARTIALLY TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -1180,7 +1181,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>PARTIALLY TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -1195,7 +1196,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>PARTIALLY TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -1210,7 +1211,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>PARTIALLY TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -1225,7 +1226,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>PARTIALLY TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -1240,7 +1241,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>PARTIALLY TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -1255,7 +1256,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>PARTIALLY TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -1270,7 +1271,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>PARTIALLY TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -1285,7 +1286,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>PARTIALLY TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -1300,7 +1301,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>PARTIALLY TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -1315,7 +1316,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>PARTIALLY TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -1330,7 +1331,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>PARTIALLY TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -1345,7 +1346,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>PARTIALLY TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -1360,7 +1361,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>PARTIALLY TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -1375,7 +1376,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>PARTIALLY TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -1390,7 +1391,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>PARTIALLY TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -1405,7 +1406,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>PARTIALLY TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -1420,7 +1421,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>PARTIALLY TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -1435,7 +1436,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>PARTIALLY TRUE</t>
+          <t>UNVERIFIABLE</t>
         </is>
       </c>
     </row>
@@ -1450,7 +1451,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>PARTIALLY TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -1465,7 +1466,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>PARTIALLY TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -1480,7 +1481,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>PARTIALLY TRUE</t>
+          <t>UNVERIFIABLE</t>
         </is>
       </c>
     </row>
@@ -1495,7 +1496,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>PARTIALLY TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -1510,7 +1511,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>PARTIALLY TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -1525,7 +1526,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>PARTIALLY TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -1540,7 +1541,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>PARTIALLY TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -1555,7 +1556,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>PARTIALLY TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -1570,7 +1571,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>PARTIALLY TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -1585,7 +1586,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>PARTIALLY TRUE</t>
+          <t>UNVERIFIABLE</t>
         </is>
       </c>
     </row>
@@ -1600,7 +1601,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>PARTIALLY TRUE</t>
+          <t>UNVERIFIABLE</t>
         </is>
       </c>
     </row>
@@ -1615,7 +1616,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>PARTIALLY TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -1630,7 +1631,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>PARTIALLY TRUE</t>
+          <t>UNVERIFIABLE</t>
         </is>
       </c>
     </row>
@@ -1645,7 +1646,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>PARTIALLY TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -1660,7 +1661,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>PARTIALLY TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -1675,7 +1676,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>PARTIALLY TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -2106,7 +2107,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2133,7 +2134,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Relevant evidence clearly confirms the claim as stated.</t>
+          <t>Evidence supports the central claim.</t>
         </is>
       </c>
     </row>
@@ -2145,31 +2146,860 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Relevant evidence clearly contradicts the claim.</t>
+          <t>Evidence contradicts the central claim (including overstated or universal wording whose core assertion is refuted).</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>PARTIALLY TRUE</t>
+          <t>UNVERIFIABLE</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Mixed evidence: some elements are accurate, but the claim overstates, omits key context, holds only under specific conditions, or creates a false impression (includes former MISLEADING).</t>
+          <t>Evidence is insufficient, inconclusive, or unavailable.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D41"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="90" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Claim_ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Previous_Label</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>New_Label</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>41</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>The Great Wall of China is visible from space.</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>42</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Humans use only 10 percent of their brains.</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>43</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Drinking eight glasses of water every day is necessary for everyone.</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" t="n">
+        <v>44</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>The Mediterranean diet prevents all heart disease.</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>45</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Vitamin C completely prevents the common cold.</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>46</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>The full moon causes people to behave more irrationally.</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>47</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Eating carrots gives you night vision.</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>48</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Coffee always causes dehydration.</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>49</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Sugar directly causes hyperactivity in every child.</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>50</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Cracking your knuckles causes arthritis.</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>51</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Cold weather itself causes the common cold.</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>52</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>An apple a day guarantees that you will never need a doctor.</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>53</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Organic food is always more nutritious than conventional food.</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>54</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Humans lose most of their body heat through their heads.</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>55</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>The five-second rule means food is safe to eat after being dropped briefly.</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>56</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Eating spicy food permanently damages the stomach.</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>57</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>A high-protein diet is always the best diet for weight loss.</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>58</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>All fats are unhealthy and should be avoided.</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>59</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Antibiotics can cure viral infections.</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>60</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Exercise can completely eliminate the risk of developing heart disease.</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>61</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>A food label says a product is fat-free, so eating unlimited amounts cannot contribute to weight gain.</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>62</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>A study found that a supplement improved memory, proving that the supplement makes everyone smarter.</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>63</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>A city experienced record rainfall this year, proving that climate change is the sole cause of that event.</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>64</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>A person recovered after taking a particular medicine, proving that the medicine caused the recovery.</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
         <is>
           <t>UNVERIFIABLE</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>No relevant sources, or insufficient information to judge.</t>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>65</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>A product contains a natural ingredient, so it is automatically safer than synthetic alternatives.</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>66</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>A vaccine was followed by a health event, proving that the vaccine caused the event.</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>67</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>A company reports that its product is used by millions, proving that it is the most effective product available.</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>UNVERIFIABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>68</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>A country has a higher GDP than another country, so every person in that country must be wealthier.</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>69</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>A news headline says temperatures are falling this week, proving that global warming has stopped.</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>70</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>A person has no symptoms, so they definitely cannot have an infectious disease.</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>71</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>A supplement is sold without a prescription, so it must be completely risk-free.</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>72</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>A graph shows two variables rising together, proving that one variable caused the other.</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>73</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>A scientific paper reports an association, proving that the observed factor directly caused the outcome.</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>74</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>A technology company has the largest market value, so its technology must be objectively the best.</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>UNVERIFIABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>75</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>A person lost weight after removing one food from their diet, proving that food is the cause of weight gain for everyone.</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>UNVERIFIABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>76</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>A historical event happened after another event, proving that the first event caused the second.</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>77</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>A product has more features than a competitor, so it must provide better value for every customer.</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>UNVERIFIABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>78</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>A single unusual weather event proves that long-term climate trends are incorrect.</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>79</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>A celebrity endorses a treatment, so the treatment must be medically effective.</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>80</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>A treatment works for one patient, proving that it will work for all patients.</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>PARTIALLY TRUE</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>FALSE</t>
         </is>
       </c>
     </row>

</xml_diff>